<commit_message>
added turn end triggers
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipi\Downloads\mtg\mtg_clone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjol\Documents\GitHub\mtg_clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6C26CE-D871-4CF4-BEAB-4452E2C739F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4B9AAE7C-4929-4CFC-9ABD-C6251723E409}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -273,8 +272,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -649,19 +648,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C0F7F3C-0E7B-406E-9B99-22B8FA879FD3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5703125" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="39.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.59765625" customWidth="1"/>
+    <col min="3" max="3" width="17.8984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.8984375" customWidth="1"/>
+    <col min="5" max="5" width="39.69921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -675,7 +674,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -691,11 +690,14 @@
       <c r="E2" t="s">
         <v>31</v>
       </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
       <c r="G2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>66</v>
       </c>
@@ -705,14 +707,20 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
       <c r="E3" t="s">
         <v>32</v>
       </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
       <c r="G3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -722,6 +730,9 @@
       <c r="C4" t="s">
         <v>14</v>
       </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
       <c r="E4" t="s">
         <v>33</v>
       </c>
@@ -729,7 +740,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -746,7 +757,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -763,7 +774,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -780,7 +791,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -794,7 +805,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -808,7 +819,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -822,7 +833,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -836,7 +847,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -850,7 +861,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -861,7 +872,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -872,7 +883,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -883,7 +894,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -894,7 +905,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -905,7 +916,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -916,7 +927,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -927,7 +938,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -938,7 +949,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -949,12 +960,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -968,9 +979,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3089236-C12C-4CAD-B4C4-6F7FBD429364}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
corrected spelling and mana movement
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipi\Downloads\mtg\mtg_clone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arjol\Documents\GitHub\mtg_clone\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B064B773-1531-48E4-8CE7-E72889B441B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>target_spec</t>
   </si>
@@ -257,13 +256,19 @@
   </si>
   <si>
     <t>none</t>
+  </si>
+  <si>
+    <t>on_end_phase_on_field</t>
+  </si>
+  <si>
+    <t>on_turn_end_on_field</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -638,19 +643,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5703125" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="39.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.59765625" customWidth="1"/>
+    <col min="3" max="3" width="20.296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.8984375" customWidth="1"/>
+    <col min="5" max="5" width="39.69921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -664,7 +669,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -687,7 +692,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -710,7 +715,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>74</v>
       </c>
@@ -730,7 +735,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -747,7 +752,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -764,7 +769,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -781,7 +786,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -795,7 +800,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -809,7 +814,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>75</v>
       </c>
@@ -823,7 +828,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -837,7 +842,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -851,7 +856,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -862,7 +867,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -873,7 +878,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>76</v>
       </c>
@@ -884,7 +889,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -895,7 +900,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -906,7 +911,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -917,7 +922,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -928,7 +933,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>47</v>
       </c>
@@ -939,7 +944,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -950,14 +955,20 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>50</v>
+      </c>
+      <c r="C23" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -969,9 +980,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>